<commit_message>
feat(ipa): rimuovi colonna N° MEMBRANA dal foglio campagna ufficiale
Rimuove colonna H "N° MEMBRANA" dal template IPA (shift I→H … L→K,
NUM_COLS 12→11). In exportSchemas.ts: rimosso mapping numero_membrana→H,
shift pompa→H, portata_q→I, durata_prelievo→J, volume_campionato→K,
strumento footer H→G.
Campo numero_membrana resta in dati e in MisuraIpaModal (non esportato).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/ipa.xlsx
+++ b/public/templates/ipa.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Foglio1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Foglio1'!$A$1:$L$52</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Foglio1'!$A$1:$K$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -491,11 +491,10 @@
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -573,27 +572,22 @@
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>N° MEMBRANA</t>
+          <t>POMPA</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>POMPA</t>
-        </is>
-      </c>
-      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>PORTATA Q
 (L/min)</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>DURATA
 (min)</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="K3" s="5" t="inlineStr">
         <is>
           <t>VOLUME
 (L)</t>
@@ -614,7 +608,6 @@
       <c r="I4" s="7" t="n"/>
       <c r="J4" s="7" t="n"/>
       <c r="K4" s="7" t="n"/>
-      <c r="L4" s="7" t="n"/>
     </row>
     <row r="5" ht="36" customHeight="1">
       <c r="A5" s="6" t="n">
@@ -630,7 +623,6 @@
       <c r="I5" s="7" t="n"/>
       <c r="J5" s="7" t="n"/>
       <c r="K5" s="7" t="n"/>
-      <c r="L5" s="7" t="n"/>
     </row>
     <row r="6" ht="36" customHeight="1">
       <c r="A6" s="6" t="n">
@@ -646,7 +638,6 @@
       <c r="I6" s="7" t="n"/>
       <c r="J6" s="7" t="n"/>
       <c r="K6" s="7" t="n"/>
-      <c r="L6" s="7" t="n"/>
     </row>
     <row r="7" ht="36" customHeight="1">
       <c r="A7" s="6" t="n">
@@ -662,7 +653,6 @@
       <c r="I7" s="7" t="n"/>
       <c r="J7" s="7" t="n"/>
       <c r="K7" s="7" t="n"/>
-      <c r="L7" s="7" t="n"/>
     </row>
     <row r="8" ht="36" customHeight="1">
       <c r="A8" s="6" t="n">
@@ -678,7 +668,6 @@
       <c r="I8" s="7" t="n"/>
       <c r="J8" s="7" t="n"/>
       <c r="K8" s="7" t="n"/>
-      <c r="L8" s="7" t="n"/>
     </row>
     <row r="9" ht="36" customHeight="1">
       <c r="A9" s="6" t="n">
@@ -694,7 +683,6 @@
       <c r="I9" s="7" t="n"/>
       <c r="J9" s="7" t="n"/>
       <c r="K9" s="7" t="n"/>
-      <c r="L9" s="7" t="n"/>
     </row>
     <row r="10" ht="36" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -710,7 +698,6 @@
       <c r="I10" s="7" t="n"/>
       <c r="J10" s="7" t="n"/>
       <c r="K10" s="7" t="n"/>
-      <c r="L10" s="7" t="n"/>
     </row>
     <row r="11" ht="36" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -726,7 +713,6 @@
       <c r="I11" s="7" t="n"/>
       <c r="J11" s="7" t="n"/>
       <c r="K11" s="7" t="n"/>
-      <c r="L11" s="7" t="n"/>
     </row>
     <row r="12" ht="27.75" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
@@ -735,7 +721,7 @@
         </is>
       </c>
       <c r="C12" s="9" t="n"/>
-      <c r="H12" s="10" t="inlineStr">
+      <c r="G12" s="10" t="inlineStr">
         <is>
           <t>Strumentazione:</t>
         </is>
@@ -817,27 +803,22 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>N° MEMBRANA</t>
+          <t>POMPA</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
-        <is>
-          <t>POMPA</t>
-        </is>
-      </c>
-      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>PORTATA Q
 (L/min)</t>
         </is>
       </c>
-      <c r="K16" s="5" t="inlineStr">
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>DURATA
 (min)</t>
         </is>
       </c>
-      <c r="L16" s="5" t="inlineStr">
+      <c r="K16" s="5" t="inlineStr">
         <is>
           <t>VOLUME
 (L)</t>
@@ -858,7 +839,6 @@
       <c r="I17" s="7" t="n"/>
       <c r="J17" s="7" t="n"/>
       <c r="K17" s="7" t="n"/>
-      <c r="L17" s="7" t="n"/>
     </row>
     <row r="18" ht="36" customHeight="1">
       <c r="A18" s="6" t="n">
@@ -874,7 +854,6 @@
       <c r="I18" s="7" t="n"/>
       <c r="J18" s="7" t="n"/>
       <c r="K18" s="7" t="n"/>
-      <c r="L18" s="7" t="n"/>
     </row>
     <row r="19" ht="36" customHeight="1">
       <c r="A19" s="6" t="n">
@@ -890,7 +869,6 @@
       <c r="I19" s="7" t="n"/>
       <c r="J19" s="7" t="n"/>
       <c r="K19" s="7" t="n"/>
-      <c r="L19" s="7" t="n"/>
     </row>
     <row r="20" ht="36" customHeight="1">
       <c r="A20" s="6" t="n">
@@ -906,7 +884,6 @@
       <c r="I20" s="7" t="n"/>
       <c r="J20" s="7" t="n"/>
       <c r="K20" s="7" t="n"/>
-      <c r="L20" s="7" t="n"/>
     </row>
     <row r="21" ht="36" customHeight="1">
       <c r="A21" s="6" t="n">
@@ -922,7 +899,6 @@
       <c r="I21" s="7" t="n"/>
       <c r="J21" s="7" t="n"/>
       <c r="K21" s="7" t="n"/>
-      <c r="L21" s="7" t="n"/>
     </row>
     <row r="22" ht="36" customHeight="1">
       <c r="A22" s="6" t="n">
@@ -938,7 +914,6 @@
       <c r="I22" s="7" t="n"/>
       <c r="J22" s="7" t="n"/>
       <c r="K22" s="7" t="n"/>
-      <c r="L22" s="7" t="n"/>
     </row>
     <row r="23" ht="36" customHeight="1">
       <c r="A23" s="6" t="n">
@@ -954,7 +929,6 @@
       <c r="I23" s="7" t="n"/>
       <c r="J23" s="7" t="n"/>
       <c r="K23" s="7" t="n"/>
-      <c r="L23" s="7" t="n"/>
     </row>
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="6" t="n">
@@ -970,7 +944,6 @@
       <c r="I24" s="7" t="n"/>
       <c r="J24" s="7" t="n"/>
       <c r="K24" s="7" t="n"/>
-      <c r="L24" s="7" t="n"/>
     </row>
     <row r="25" ht="27.75" customHeight="1">
       <c r="A25" s="8" t="inlineStr">
@@ -979,7 +952,7 @@
         </is>
       </c>
       <c r="C25" s="9" t="n"/>
-      <c r="H25" s="10" t="inlineStr">
+      <c r="G25" s="10" t="inlineStr">
         <is>
           <t>Strumentazione:</t>
         </is>
@@ -1061,27 +1034,22 @@
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>N° MEMBRANA</t>
+          <t>POMPA</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
-        <is>
-          <t>POMPA</t>
-        </is>
-      </c>
-      <c r="J29" s="5" t="inlineStr">
         <is>
           <t>PORTATA Q
 (L/min)</t>
         </is>
       </c>
-      <c r="K29" s="5" t="inlineStr">
+      <c r="J29" s="5" t="inlineStr">
         <is>
           <t>DURATA
 (min)</t>
         </is>
       </c>
-      <c r="L29" s="5" t="inlineStr">
+      <c r="K29" s="5" t="inlineStr">
         <is>
           <t>VOLUME
 (L)</t>
@@ -1102,7 +1070,6 @@
       <c r="I30" s="7" t="n"/>
       <c r="J30" s="7" t="n"/>
       <c r="K30" s="7" t="n"/>
-      <c r="L30" s="7" t="n"/>
     </row>
     <row r="31" ht="36" customHeight="1">
       <c r="A31" s="6" t="n">
@@ -1118,7 +1085,6 @@
       <c r="I31" s="7" t="n"/>
       <c r="J31" s="7" t="n"/>
       <c r="K31" s="7" t="n"/>
-      <c r="L31" s="7" t="n"/>
     </row>
     <row r="32" ht="36" customHeight="1">
       <c r="A32" s="6" t="n">
@@ -1134,7 +1100,6 @@
       <c r="I32" s="7" t="n"/>
       <c r="J32" s="7" t="n"/>
       <c r="K32" s="7" t="n"/>
-      <c r="L32" s="7" t="n"/>
     </row>
     <row r="33" ht="36" customHeight="1">
       <c r="A33" s="6" t="n">
@@ -1150,7 +1115,6 @@
       <c r="I33" s="7" t="n"/>
       <c r="J33" s="7" t="n"/>
       <c r="K33" s="7" t="n"/>
-      <c r="L33" s="7" t="n"/>
     </row>
     <row r="34" ht="36" customHeight="1">
       <c r="A34" s="6" t="n">
@@ -1166,7 +1130,6 @@
       <c r="I34" s="7" t="n"/>
       <c r="J34" s="7" t="n"/>
       <c r="K34" s="7" t="n"/>
-      <c r="L34" s="7" t="n"/>
     </row>
     <row r="35" ht="36" customHeight="1">
       <c r="A35" s="6" t="n">
@@ -1182,7 +1145,6 @@
       <c r="I35" s="7" t="n"/>
       <c r="J35" s="7" t="n"/>
       <c r="K35" s="7" t="n"/>
-      <c r="L35" s="7" t="n"/>
     </row>
     <row r="36" ht="36" customHeight="1">
       <c r="A36" s="6" t="n">
@@ -1198,7 +1160,6 @@
       <c r="I36" s="7" t="n"/>
       <c r="J36" s="7" t="n"/>
       <c r="K36" s="7" t="n"/>
-      <c r="L36" s="7" t="n"/>
     </row>
     <row r="37" ht="36" customHeight="1">
       <c r="A37" s="6" t="n">
@@ -1214,7 +1175,6 @@
       <c r="I37" s="7" t="n"/>
       <c r="J37" s="7" t="n"/>
       <c r="K37" s="7" t="n"/>
-      <c r="L37" s="7" t="n"/>
     </row>
     <row r="38" ht="27.75" customHeight="1">
       <c r="A38" s="8" t="inlineStr">
@@ -1223,7 +1183,7 @@
         </is>
       </c>
       <c r="C38" s="9" t="n"/>
-      <c r="H38" s="10" t="inlineStr">
+      <c r="G38" s="10" t="inlineStr">
         <is>
           <t>Strumentazione:</t>
         </is>
@@ -1305,27 +1265,22 @@
       </c>
       <c r="H42" s="5" t="inlineStr">
         <is>
-          <t>N° MEMBRANA</t>
+          <t>POMPA</t>
         </is>
       </c>
       <c r="I42" s="5" t="inlineStr">
-        <is>
-          <t>POMPA</t>
-        </is>
-      </c>
-      <c r="J42" s="5" t="inlineStr">
         <is>
           <t>PORTATA Q
 (L/min)</t>
         </is>
       </c>
-      <c r="K42" s="5" t="inlineStr">
+      <c r="J42" s="5" t="inlineStr">
         <is>
           <t>DURATA
 (min)</t>
         </is>
       </c>
-      <c r="L42" s="5" t="inlineStr">
+      <c r="K42" s="5" t="inlineStr">
         <is>
           <t>VOLUME
 (L)</t>
@@ -1346,7 +1301,6 @@
       <c r="I43" s="7" t="n"/>
       <c r="J43" s="7" t="n"/>
       <c r="K43" s="7" t="n"/>
-      <c r="L43" s="7" t="n"/>
     </row>
     <row r="44" ht="36" customHeight="1">
       <c r="A44" s="6" t="n">
@@ -1362,7 +1316,6 @@
       <c r="I44" s="7" t="n"/>
       <c r="J44" s="7" t="n"/>
       <c r="K44" s="7" t="n"/>
-      <c r="L44" s="7" t="n"/>
     </row>
     <row r="45" ht="36" customHeight="1">
       <c r="A45" s="6" t="n">
@@ -1378,7 +1331,6 @@
       <c r="I45" s="7" t="n"/>
       <c r="J45" s="7" t="n"/>
       <c r="K45" s="7" t="n"/>
-      <c r="L45" s="7" t="n"/>
     </row>
     <row r="46" ht="36" customHeight="1">
       <c r="A46" s="6" t="n">
@@ -1394,7 +1346,6 @@
       <c r="I46" s="7" t="n"/>
       <c r="J46" s="7" t="n"/>
       <c r="K46" s="7" t="n"/>
-      <c r="L46" s="7" t="n"/>
     </row>
     <row r="47" ht="36" customHeight="1">
       <c r="A47" s="6" t="n">
@@ -1410,7 +1361,6 @@
       <c r="I47" s="7" t="n"/>
       <c r="J47" s="7" t="n"/>
       <c r="K47" s="7" t="n"/>
-      <c r="L47" s="7" t="n"/>
     </row>
     <row r="48" ht="36" customHeight="1">
       <c r="A48" s="6" t="n">
@@ -1426,7 +1376,6 @@
       <c r="I48" s="7" t="n"/>
       <c r="J48" s="7" t="n"/>
       <c r="K48" s="7" t="n"/>
-      <c r="L48" s="7" t="n"/>
     </row>
     <row r="49" ht="36" customHeight="1">
       <c r="A49" s="6" t="n">
@@ -1442,7 +1391,6 @@
       <c r="I49" s="7" t="n"/>
       <c r="J49" s="7" t="n"/>
       <c r="K49" s="7" t="n"/>
-      <c r="L49" s="7" t="n"/>
     </row>
     <row r="50" ht="36" customHeight="1">
       <c r="A50" s="6" t="n">
@@ -1458,7 +1406,6 @@
       <c r="I50" s="7" t="n"/>
       <c r="J50" s="7" t="n"/>
       <c r="K50" s="7" t="n"/>
-      <c r="L50" s="7" t="n"/>
     </row>
     <row r="51" ht="27.75" customHeight="1">
       <c r="A51" s="8" t="inlineStr">
@@ -1467,7 +1414,7 @@
         </is>
       </c>
       <c r="C51" s="9" t="n"/>
-      <c r="H51" s="10" t="inlineStr">
+      <c r="G51" s="10" t="inlineStr">
         <is>
           <t>Strumentazione:</t>
         </is>
@@ -1476,34 +1423,34 @@
     <row r="52" ht="15" customHeight="1"/>
   </sheetData>
   <mergeCells count="28">
-    <mergeCell ref="A41:L41"/>
-    <mergeCell ref="H38:L38"/>
+    <mergeCell ref="G12:K12"/>
+    <mergeCell ref="A15:K15"/>
     <mergeCell ref="J14:K14"/>
     <mergeCell ref="A51:B51"/>
     <mergeCell ref="J1:K1"/>
+    <mergeCell ref="C38:F38"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="J40:K40"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="H25:L25"/>
     <mergeCell ref="A25:B25"/>
     <mergeCell ref="F27:H27"/>
-    <mergeCell ref="H51:L51"/>
-    <mergeCell ref="C25:G25"/>
+    <mergeCell ref="G38:K38"/>
+    <mergeCell ref="A41:K41"/>
     <mergeCell ref="B14:C14"/>
     <mergeCell ref="J27:K27"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="A12:B12"/>
-    <mergeCell ref="C12:G12"/>
     <mergeCell ref="F14:H14"/>
     <mergeCell ref="F1:H1"/>
-    <mergeCell ref="A28:L28"/>
-    <mergeCell ref="C51:G51"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="C25:F25"/>
     <mergeCell ref="B40:C40"/>
     <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A15:L15"/>
-    <mergeCell ref="H12:L12"/>
-    <mergeCell ref="C38:G38"/>
+    <mergeCell ref="G51:K51"/>
+    <mergeCell ref="C12:F12"/>
+    <mergeCell ref="G25:K25"/>
     <mergeCell ref="F40:H40"/>
+    <mergeCell ref="A28:K28"/>
+    <mergeCell ref="C51:F51"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>

</xml_diff>